<commit_message>
fix diersity metrics code
</commit_message>
<xml_diff>
--- a/Tabla parametros escenarios.xlsx
+++ b/Tabla parametros escenarios.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/catg/Desktop/SOFIAC/TESIS MAGISTER/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/catg/Desktop/SOFIAC/Gitsofia/tesisbioinf-sofia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BD77DA4-7F72-F748-BC35-325728B07B93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EC7CE18-31B0-FA48-95D3-C74353ECB951}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="26400" yWindow="1080" windowWidth="24800" windowHeight="17440" xr2:uid="{412D9DDC-1BB5-C942-ABB5-185C869803BA}"/>
   </bookViews>
@@ -413,7 +413,7 @@
   </si>
   <si>
     <r>
-      <t>Bajo data (prob 15/350 / 5%)</t>
+      <t>Bajo data (prob 20/350 / 5%)</t>
     </r>
     <r>
       <rPr>

</xml_diff>